<commit_message>
fix(exporter-gm): benchmark default 35% para PEPs Apps sem pessoas
Apps não estava em WS_MB_BENCHMARK (só cloud/dados/hyper/demais).
Agora aplica 35% default quando receita > 0 e custo = 0, mesmo fallback
do engine. Elimina as 8 linhas com custo zerado no arquivo.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/grupo_mult_q4.xlsx
+++ b/backend/grupo_mult_q4.xlsx
@@ -1789,13 +1789,13 @@
         <v>124297.64</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>0</v>
+        <v>-80793.466</v>
       </c>
       <c r="L23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>124297.64</v>
+        <v>43504.174</v>
       </c>
     </row>
     <row r="24">
@@ -1966,13 +1966,13 @@
         <v>46556.48</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>-30261.712</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>46556.48</v>
+        <v>16294.768</v>
       </c>
     </row>
     <row r="27">
@@ -3075,13 +3075,13 @@
         <v>2011.2</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>0</v>
+        <v>-1307.28</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>2011.2</v>
+        <v>703.9200000000001</v>
       </c>
     </row>
     <row r="46">
@@ -3523,13 +3523,13 @@
         <v>14427.93</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0</v>
+        <v>-9378.154500000001</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>14427.93</v>
+        <v>5049.7755</v>
       </c>
     </row>
     <row r="54">
@@ -3578,13 +3578,13 @@
         <v>14427.93</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0</v>
+        <v>-9378.154500000001</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>14427.93</v>
+        <v>5049.7755</v>
       </c>
     </row>
     <row r="55">
@@ -3633,13 +3633,13 @@
         <v>14427.93</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0</v>
+        <v>-9378.154500000001</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>14427.93</v>
+        <v>5049.7755</v>
       </c>
     </row>
     <row r="56">
@@ -3916,13 +3916,13 @@
         <v>34849.40999999999</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0</v>
+        <v>-22652.11649999999</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>34849.40999999999</v>
+        <v>12197.2935</v>
       </c>
     </row>
     <row r="61">
@@ -3975,13 +3975,13 @@
         <v>42089.24999999999</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0</v>
+        <v>-27358.0125</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>42089.24999999999</v>
+        <v>14731.2375</v>
       </c>
     </row>
     <row r="62">

</xml_diff>

<commit_message>
fix(exporter-gm): atribui AE para variantes do SAP sem cadastro exato
Override no arquivo grupo_mult_q4.xlsx (mesmo mapeamento do engine):
- DIRECIONAL ENGENHARIA S/A -> Guilherme
- UNIMED BELO HORIZONTE COOPERATIVA D -> Danilo
- LOJA ELETRICA LTDA -> Danilo

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/grupo_mult_q4.xlsx
+++ b/backend/grupo_mult_q4.xlsx
@@ -1418,7 +1418,11 @@
           <t>DIRECIONAL ENGENHARIA S/A</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>GUILHERME</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>Taxa hora - Time and Expenses</t>
@@ -1473,7 +1477,11 @@
           <t>DIRECIONAL ENGENHARIA S/A</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>GUILHERME</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>Taxa hora - Time and Expenses</t>
@@ -1528,7 +1536,11 @@
           <t>DIRECIONAL ENGENHARIA S/A</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>GUILHERME</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>Taxa hora - Time and Expenses</t>
@@ -3498,7 +3510,11 @@
           <t>UNIMED BELO HORIZONTE COOPERATIVA D</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>DANILO DE SOUZA MACIEIRA</t>
+        </is>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>Fee</t>
@@ -3553,7 +3569,11 @@
           <t>UNIMED BELO HORIZONTE COOPERATIVA D</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>DANILO DE SOUZA MACIEIRA</t>
+        </is>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>Fee</t>
@@ -3608,7 +3628,11 @@
           <t>UNIMED BELO HORIZONTE COOPERATIVA D</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>DANILO DE SOUZA MACIEIRA</t>
+        </is>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>Fee</t>
@@ -12030,7 +12054,11 @@
           <t>DIRECIONAL ENGENHARIA S/A</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>GUILHERME</t>
+        </is>
+      </c>
       <c r="F179" t="inlineStr">
         <is>
           <t>Rian  Goetz Pasquali</t>
@@ -12067,7 +12095,11 @@
           <t>DIRECIONAL ENGENHARIA S/A</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>GUILHERME</t>
+        </is>
+      </c>
       <c r="F180" t="inlineStr">
         <is>
           <t>RIAN GOETZ PASQUALI</t>
@@ -12104,7 +12136,11 @@
           <t>DIRECIONAL ENGENHARIA S/A</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>GUILHERME</t>
+        </is>
+      </c>
       <c r="F181" t="inlineStr">
         <is>
           <t>RIAN GOETZ PASQUALI</t>

</xml_diff>

<commit_message>
fix(q4): BR02CLP00035 dez Klabin remove rec R$87.370 / custo R$43.685
Ajuste em exporter e engine para consistencia Q3/Q4.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/grupo_mult_q4.xlsx
+++ b/backend/grupo_mult_q4.xlsx
@@ -1739,16 +1739,16 @@
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>986660.9300000001</v>
+        <v>899290.79</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>-142560.3855865922</v>
+        <v>-98875.31558659219</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>1072</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>844100.5444134078</v>
+        <v>800415.4744134079</v>
       </c>
     </row>
     <row r="23">

</xml_diff>